<commit_message>
Write Excel file added
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -189,9 +189,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0;[Red]0"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="6">
     <font>
       <sz val="11.0"/>
@@ -345,28 +343,28 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="true" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="1" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="true" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="true"/>

</xml_diff>

<commit_message>
Hyperlinks to libraries added
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -189,7 +189,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0;[Red]0"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <sz val="11.0"/>
@@ -343,28 +345,28 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="true" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="true" applyFill="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="true"/>

</xml_diff>